<commit_message>
add branch data ti student file
</commit_message>
<xml_diff>
--- a/student-data.xlsx
+++ b/student-data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8808ff2ef71e9856/Documents/Desktop/git_and_github_practice/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_F25DC773A252ABDACC104860D19949345ADE58E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC5A1ACB-DDFE-4E3C-94AD-34503BDA0E39}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="11_F25DC773A252ABDACC104860D19949345ADE58E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FEF8AAE0-CA72-4361-B1CF-0C4E6226B7F9}"/>
   <bookViews>
     <workbookView xWindow="795" yWindow="2085" windowWidth="15375" windowHeight="8715" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>NAME</t>
   </si>
@@ -37,6 +37,12 @@
   </si>
   <si>
     <t>PYTHON</t>
+  </si>
+  <si>
+    <t>DEPT</t>
+  </si>
+  <si>
+    <t>AIDS</t>
   </si>
 </sst>
 </file>
@@ -98,6 +104,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -364,7 +374,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -383,6 +393,14 @@
         <v>3</v>
       </c>
     </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>